<commit_message>
Data migration data cleaning files
</commit_message>
<xml_diff>
--- a/src/CJMSS.DataMigration/Migration Data Files/StockCategory.xlsx
+++ b/src/CJMSS.DataMigration/Migration Data Files/StockCategory.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yorgoinc.sharepoint.com/sites/PurpleDigitsProjects/Shared Documents/Jewelry Management System - JMS/Git/CJMSS/docs/Migration Data Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yorgoinc.sharepoint.com/sites/PurpleDigitsProjects/Shared Documents/Jewelry Management System - JMS/Git/CJMSS/src/CJMSS.DataMigration/Migration Data Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{60C6A082-5926-406D-9C5B-FC882E48B4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{60C6A082-5926-406D-9C5B-FC882E48B4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B47D0D18-6D46-4895-A924-8E7F44213533}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4524,6 +4524,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D353"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.1796875" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" customWidth="1"/>
+    <col min="3" max="3" width="16.26953125" customWidth="1"/>
+    <col min="4" max="4" width="22.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -9473,6 +9479,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8db5f02f-16cf-417c-b8d5-ebbf7ea068b2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a7dd6fdb-24d5-4f36-9343-ebf87e8a3b8a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A4FB4374F3262F4DAB3E5936217975C0" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9ec3ae9ae41c6a02cc9ee16082b2f8e4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a7dd6fdb-24d5-4f36-9343-ebf87e8a3b8a" xmlns:ns3="8db5f02f-16cf-417c-b8d5-ebbf7ea068b2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="45ef9aee5f347cbd41fbbf5d6a6bb7eb" ns2:_="" ns3:_="">
     <xsd:import namespace="a7dd6fdb-24d5-4f36-9343-ebf87e8a3b8a"/>
@@ -9701,34 +9727,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="8db5f02f-16cf-417c-b8d5-ebbf7ea068b2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a7dd6fdb-24d5-4f36-9343-ebf87e8a3b8a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{421AE1A8-B6E4-4EB8-B431-A606865F1008}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{839BA1E8-A723-41D2-A156-162914B134D6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8db5f02f-16cf-417c-b8d5-ebbf7ea068b2"/>
+    <ds:schemaRef ds:uri="a7dd6fdb-24d5-4f36-9343-ebf87e8a3b8a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF6BE004-9E4E-4076-8DDC-BF4D05F24FF8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF6BE004-9E4E-4076-8DDC-BF4D05F24FF8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{839BA1E8-A723-41D2-A156-162914B134D6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{421AE1A8-B6E4-4EB8-B431-A606865F1008}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a7dd6fdb-24d5-4f36-9343-ebf87e8a3b8a"/>
+    <ds:schemaRef ds:uri="8db5f02f-16cf-417c-b8d5-ebbf7ea068b2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>